<commit_message>
Give the cluster sampling dataset the American wording its notebook shows
The workbook's plan, codebook, notes and truth sheets said "Year 6", "state schools" and "roll",
while the notebook's saved output read sixth-grade and public schools, so a fresh run printed the
British text. The sheets now say sixth-grade, public schools and enrollment, the notes call the
simulated truth the true population values, and the chapter and notebook say enrollment for roll.
</commit_message>
<xml_diff>
--- a/data/capstone-cluster-sampling-schools.xlsx
+++ b/data/capstone-cluster-sampling-schools.xlsx
@@ -16576,7 +16576,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Year 6 students</t>
+          <t>sixth-grade students</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -16610,14 +16610,14 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>D1 TARGET POPULATION: all Year 6 students in the district's 120 state schools.</t>
+          <t>D1 TARGET POPULATION: all sixth-grade students in the district's 120 public schools.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>D2 FRAME: there is NO central list of students. There IS a complete list of schools, with roll</t>
+          <t>D2 FRAME: there is NO central list of students. There IS a complete list of schools, with enrollment</t>
         </is>
       </c>
     </row>
@@ -16638,7 +16638,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Stage 2 draws 25 Year 6 students at random within each selected school. n = 600 students.</t>
+          <t xml:space="preserve">   Stage 2 draws 25 sixth-grade students at random within each selected school. n = 600 students.</t>
         </is>
       </c>
     </row>
@@ -16795,7 +16795,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Year 6 roll at that school, from the frame.</t>
+          <t>Sixth-grade enrollment at that school, from the frame.</t>
         </is>
       </c>
     </row>
@@ -16877,7 +16877,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>A two-stage cluster sample: 24 schools drawn from 120, then 25 Year 6 students within each.</t>
+          <t>A two-stage cluster sample: 24 schools drawn from 120, then 25 sixth-grade students within each.</t>
         </is>
       </c>
     </row>
@@ -16898,7 +16898,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>The 'truth' sheet holds the real population values, available only because the population is</t>
+          <t>The 'truth' sheet holds the true population values, available only because the population is</t>
         </is>
       </c>
     </row>

</xml_diff>